<commit_message>
updating test scenario and test case
</commit_message>
<xml_diff>
--- a/docs/test case.xlsx
+++ b/docs/test case.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="89">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -199,17 +199,6 @@
   </si>
   <si>
     <t>TS11</t>
-  </si>
-  <si>
-    <t>Provera da li su usluge salona prikazane na naslovnoj strani</t>
-  </si>
-  <si>
-    <t>1. Otvoriti početnu stranicu
-2. Pročitati tekst celog body elementa
-3. Proveriti da li tekst sadrži reči 'Ceragem', 'Presoterapija' i 'Kavitacija'</t>
-  </si>
-  <si>
-    <t>Nazivi usluga Ceragem, Presoterapija i Kavitacija su vidljivi na naslovnoj strani</t>
   </si>
   <si>
     <t>TC11</t>
@@ -257,9 +246,6 @@
     <t>TC15</t>
   </si>
   <si>
-    <t>TS16</t>
-  </si>
-  <si>
     <t>Provera da li robots meta tag dozvoljava indeksiranje</t>
   </si>
   <si>
@@ -272,9 +258,6 @@
     <t>Robots meta tag postoji i ne blokira indeksiranje sajta od strane pretraživača</t>
   </si>
   <si>
-    <t>TC16</t>
-  </si>
-  <si>
     <t>Provera da li hamburger meni postoji na mobilnom prikazu</t>
   </si>
   <si>
@@ -315,20 +298,29 @@
 4. Proveriti da širina stranice nije veća od viewport-a za više od 5px</t>
   </si>
   <si>
+    <t>TEST SLUČAJEVI</t>
+  </si>
+  <si>
     <t>1. Otvoriti početnu stranicu
 2. Pronaći meta tag sa atributom name='description'
 3. Pročitati vrednost content atributa
-4. Proveriti da li sadrži neku od reči: ceragem, salon, kozmetički, tretman</t>
-  </si>
-  <si>
-    <t>TEST SLUČAJEVI</t>
+4. Proveriti da li sadrži neku od reči: ceragem, salon, kozmetičk, tretman</t>
+  </si>
+  <si>
+    <t>PASSED</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>Telefon link postoji u HTML kodu stranice, ali nije vidljiv na mobilnom prikazu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -354,6 +346,32 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -417,23 +435,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -750,16 +777,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="A1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -787,361 +814,403 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-    </row>
-    <row r="4" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="G3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-    </row>
-    <row r="5" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="G4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-    </row>
-    <row r="6" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="G5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-    </row>
-    <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="G6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-    </row>
-    <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="G7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-    </row>
-    <row r="9" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="G8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-    </row>
-    <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="G9" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-    </row>
-    <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-    </row>
-    <row r="12" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-    </row>
-    <row r="13" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-    </row>
-    <row r="14" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+    </row>
+    <row r="17" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="C17" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="F16" s="5" t="s">
+      <c r="E17" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
+      <c r="G17" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>